<commit_message>
bug fix all bikes fit 176cm
</commit_message>
<xml_diff>
--- a/data/gravel/Pivot Les 2025.xlsx
+++ b/data/gravel/Pivot Les 2025.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/walker/Documents/Github/Bike Geometry Project/data/gravel/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5126CC3F-3F80-9F4B-8FAD-BD816FFEE9B2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B0A6EE98-2CE6-CA47-971C-1BD8F73D88A3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="4100" yWindow="500" windowWidth="24700" windowHeight="17500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="33040" yWindow="-20040" windowWidth="24700" windowHeight="17500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -1540,11 +1540,16 @@
       <c r="A45" t="s">
         <v>40</v>
       </c>
-      <c r="B45" s="1"/>
+      <c r="B45" s="1">
+        <v>100</v>
+      </c>
     </row>
     <row r="46" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A46" t="s">
         <v>41</v>
+      </c>
+      <c r="B46">
+        <v>100</v>
       </c>
     </row>
     <row r="47" spans="1:6" x14ac:dyDescent="0.3">

</xml_diff>